<commit_message>
Addition of to the app
Addition of new tab for project summary and locations for some projects in Ho Municipal.
</commit_message>
<xml_diff>
--- a/vrcc.xlsx
+++ b/vrcc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidackuaku/Desktop/VRCC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1F9A9E-6E58-7440-B1BD-141DEB2E98BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C2DCCFE-769C-1547-8AFF-0F976E65896D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{690D29BB-E107-B54C-8AFA-AAD6A1551766}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{690D29BB-E107-B54C-8AFA-AAD6A1551766}"/>
   </bookViews>
   <sheets>
     <sheet name="projects" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">media!$A$1:$E$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">media!$A$1:$E$30</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="139">
   <si>
     <t>District</t>
   </si>
@@ -356,6 +356,108 @@
   </si>
   <si>
     <t>First site meeting for the construction Starting for the 24 Hr Economy Market</t>
+  </si>
+  <si>
+    <t>Deme-Fiave Envlave</t>
+  </si>
+  <si>
+    <t>Kharista Road</t>
+  </si>
+  <si>
+    <t>Ho-Deme</t>
+  </si>
+  <si>
+    <t>Ho-Fiave</t>
+  </si>
+  <si>
+    <t>Ho-Adzimakofe</t>
+  </si>
+  <si>
+    <t>Culvert Construction-Some</t>
+  </si>
+  <si>
+    <t>Culvert Construction-Adzimakofe</t>
+  </si>
+  <si>
+    <t>HM006</t>
+  </si>
+  <si>
+    <t>HM007</t>
+  </si>
+  <si>
+    <t>HM008</t>
+  </si>
+  <si>
+    <t>HM009</t>
+  </si>
+  <si>
+    <t>Municipal Assembly</t>
+  </si>
+  <si>
+    <t>Three ongoing culvert construction in the Ho Municipality. Some Culvert.</t>
+  </si>
+  <si>
+    <t>Ho-Some</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791907259/HM_BRDcs003.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791907255/HM_BRDcs002.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791907256/HM_BRDcadz001.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791907260/HM_BRDcadzi003.jpg</t>
+  </si>
+  <si>
+    <t>Inspection tour conducted at the locations of the Culvert in the Municipal. Ho-Adzimakofe</t>
+  </si>
+  <si>
+    <t>Inspection tour conducted at the locations of the Culvert in the Municipality by Hon Stephen Adom and his team. Ho-Some</t>
+  </si>
+  <si>
+    <t>Inspection tour conducted at the locations of the Culvert in the Municipality by the Hon MCE and his team. Ho-Adzimakofe</t>
+  </si>
+  <si>
+    <t>Inspection tour conducted at the locations of the Culvert in the Municipality by the Hon. MCE and his team. Ho-Adzimakofe</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791907255/HM_BRDcs001.jpg</t>
+  </si>
+  <si>
+    <t>Work is steadily progressing on the road opening project within the Deme and Fiave enclaves, aimed at improving access and connectivity for residents.</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791908934/HM_RDfe001.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791908935/HM_RDfe002.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791908935/HM_RDfe003.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791908936/HM_RDfe004.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pictures of work progressing on the Deme Fiave enclaves. </t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dgclahox/image/upload/v1791907258/HM_BRDchtu002.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steady progress being made on the ongoing road opening works within the Muicipality at Barracks New Town to Kharista School and CK road. This is to improve accessibility, ease trafic flow, and support development within the municipality. Work is expected to be extended to other parts of the municipality. </t>
+  </si>
+  <si>
+    <t>Hon. MCE and his team inspecting work progress.</t>
+  </si>
+  <si>
+    <t>Hon. Ho Municipal Chief Executive and his team inspecting work progress.</t>
+  </si>
+  <si>
+    <t>Hon. Stepehn Adom, the MCE for Ho Municipal and his team inspecting work progress.</t>
   </si>
 </sst>
 </file>
@@ -439,7 +541,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -462,6 +564,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -797,7 +900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773B53BD-F917-6C4E-8253-31D0BBDF4EF2}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -805,7 +908,7 @@
     <col min="6" max="6" width="52.83203125" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" customWidth="1"/>
     <col min="11" max="11" width="18.5" customWidth="1"/>
     <col min="12" max="12" width="30" customWidth="1"/>
   </cols>
@@ -1035,6 +1138,9 @@
       <c r="I7" s="4">
         <v>46258</v>
       </c>
+      <c r="J7" s="14" t="s">
+        <v>116</v>
+      </c>
       <c r="K7" t="s">
         <v>20</v>
       </c>
@@ -1067,6 +1173,9 @@
       <c r="I8" s="4">
         <v>46275</v>
       </c>
+      <c r="J8" s="14" t="s">
+        <v>116</v>
+      </c>
       <c r="K8" t="s">
         <v>67</v>
       </c>
@@ -1096,8 +1205,136 @@
       <c r="H9" s="1" t="s">
         <v>81</v>
       </c>
+      <c r="J9" s="14" t="s">
+        <v>116</v>
+      </c>
       <c r="K9" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="85">
+      <c r="A10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10">
+        <v>6.6063000000000001</v>
+      </c>
+      <c r="E10">
+        <v>0.47189999999999999</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="G10" t="s">
+        <v>4</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J10" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="K10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="51">
+      <c r="A11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11">
+        <v>6.6037999999999997</v>
+      </c>
+      <c r="E11">
+        <v>0.46879999999999999</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="G11" t="s">
+        <v>4</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J11" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="K11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="34">
+      <c r="A12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12">
+        <v>6.6134000000000004</v>
+      </c>
+      <c r="E12">
+        <v>0.47689999999999999</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G12" t="s">
+        <v>4</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="J12" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="K12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13">
+        <v>6.6238999999999999</v>
+      </c>
+      <c r="E13">
+        <v>0.47</v>
+      </c>
+      <c r="G13" t="s">
+        <v>4</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J13" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="K13" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1108,21 +1345,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751A449C-0CEB-BA49-A044-736BF91FB682}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="89.5" customWidth="1"/>
-    <col min="3" max="3" width="75.33203125" customWidth="1"/>
+    <col min="3" max="3" width="75.33203125" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="17">
       <c r="A1" t="s">
         <v>28</v>
       </c>
       <c r="B1" t="s">
         <v>37</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="9" t="s">
         <v>38</v>
       </c>
       <c r="D1" t="s">
@@ -1183,7 +1420,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" hidden="1">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -1200,7 +1437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" hidden="1">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -1217,7 +1454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" hidden="1">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -1234,7 +1471,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" hidden="1">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1251,14 +1488,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1">
+    <row r="9" spans="1:5" ht="17">
       <c r="A9" t="s">
         <v>58</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="9" t="s">
         <v>57</v>
       </c>
       <c r="D9" t="s">
@@ -1268,14 +1505,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1">
+    <row r="10" spans="1:5" ht="17">
       <c r="A10" t="s">
         <v>58</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="9" t="s">
         <v>57</v>
       </c>
       <c r="D10" t="s">
@@ -1285,14 +1522,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1">
+    <row r="11" spans="1:5" ht="17">
       <c r="A11" t="s">
         <v>58</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="9" t="s">
         <v>57</v>
       </c>
       <c r="D11" t="s">
@@ -1302,14 +1539,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1">
+    <row r="12" spans="1:5" ht="17">
       <c r="A12" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="9" t="s">
         <v>57</v>
       </c>
       <c r="D12" t="s">
@@ -1438,7 +1675,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" hidden="1">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -1455,7 +1692,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" hidden="1">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -1472,7 +1709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" hidden="1">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -1489,7 +1726,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" hidden="1">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -1557,7 +1794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" hidden="1">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -1574,7 +1811,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" hidden="1">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -1608,11 +1845,250 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:5" ht="34">
+      <c r="A30" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D30" t="s">
+        <v>85</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="34">
+      <c r="A31" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D31" t="s">
+        <v>85</v>
+      </c>
+      <c r="E31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="34">
+      <c r="A32" t="s">
+        <v>115</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="D32" t="s">
+        <v>85</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="17">
+      <c r="A33" t="s">
+        <v>115</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" t="s">
+        <v>85</v>
+      </c>
+      <c r="E33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="34">
+      <c r="A34" t="s">
+        <v>115</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D34" t="s">
+        <v>85</v>
+      </c>
+      <c r="E34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="34">
+      <c r="A35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D35" t="s">
+        <v>85</v>
+      </c>
+      <c r="E35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="17">
+      <c r="A36" t="s">
+        <v>113</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="17">
+      <c r="A37" t="s">
+        <v>113</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D37" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="17">
+      <c r="A38" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D38" t="s">
+        <v>85</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="17">
+      <c r="A39" t="s">
+        <v>113</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D39" t="s">
+        <v>85</v>
+      </c>
+      <c r="E39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="17">
+      <c r="A40" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D40" t="s">
+        <v>85</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="17">
+      <c r="A41" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D41" t="s">
+        <v>85</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="17">
+      <c r="A42" t="s">
+        <v>112</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D42" t="s">
+        <v>85</v>
+      </c>
+      <c r="E42">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="17">
+      <c r="A43" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D43" t="s">
+        <v>85</v>
+      </c>
+      <c r="E43">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E29" xr:uid="{751A449C-0CEB-BA49-A044-736BF91FB682}">
+  <autoFilter ref="A1:E30" xr:uid="{751A449C-0CEB-BA49-A044-736BF91FB682}">
     <filterColumn colId="0">
       <filters>
-        <filter val="HM002"/>
+        <filter val="HM004"/>
+        <filter val="HM008"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -1649,6 +2125,20 @@
     <hyperlink ref="B27" r:id="rId26" xr:uid="{97819A27-9770-AC4D-AB83-857D3AB7B217}"/>
     <hyperlink ref="B28" r:id="rId27" xr:uid="{DDA6D94F-261D-3544-84CA-DD279F702337}"/>
     <hyperlink ref="B29" r:id="rId28" xr:uid="{75A335A5-E61F-5640-8B15-B4186F3FE177}"/>
+    <hyperlink ref="B31" r:id="rId29" xr:uid="{7B3A13F3-ECC7-0B4A-9EC4-77EF525F9A08}"/>
+    <hyperlink ref="B32" r:id="rId30" xr:uid="{380454CB-3E07-664D-BBF3-FE6519AF3A34}"/>
+    <hyperlink ref="B34" r:id="rId31" xr:uid="{D40024C8-F986-3446-81F9-A2C6DC1B004D}"/>
+    <hyperlink ref="B35" r:id="rId32" xr:uid="{6A2747D6-7187-2C49-8AB3-E63FBF1EE131}"/>
+    <hyperlink ref="B30" r:id="rId33" xr:uid="{EE6CF395-1421-B742-8CF9-1A809F458F52}"/>
+    <hyperlink ref="B36" r:id="rId34" xr:uid="{AA92B71D-9F59-4A40-8ADD-41B06697A5E3}"/>
+    <hyperlink ref="B37" r:id="rId35" xr:uid="{F856D732-B5AB-7B40-AF25-A2EF53E4C203}"/>
+    <hyperlink ref="B38" r:id="rId36" xr:uid="{4C1CDA3E-43A9-3240-877B-B89B95A329E8}"/>
+    <hyperlink ref="B39" r:id="rId37" xr:uid="{F425F5E7-F3F2-AF41-B006-F06BECDA154F}"/>
+    <hyperlink ref="B33" r:id="rId38" xr:uid="{1B5B4D62-A43B-6444-9FA3-D58DAEE7FBBE}"/>
+    <hyperlink ref="B40" r:id="rId39" xr:uid="{B8B92E69-40B1-C647-BFF6-D2D2DC453E15}"/>
+    <hyperlink ref="B41" r:id="rId40" xr:uid="{C0B501C6-8E13-2D45-88A6-0564576A563B}"/>
+    <hyperlink ref="B42" r:id="rId41" xr:uid="{FAA66490-C041-2D4F-9945-BF26AA110B79}"/>
+    <hyperlink ref="B43" r:id="rId42" xr:uid="{7EC83354-E347-684E-B4AC-089AA40C073F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>